<commit_message>
Add core-3 (DM/HTN/CKD) condition-specific and joint-profile RR analysis
Adds a cohort/analysis branch independent of analysis_df (03_relative_risk.R):
complete-case only on diabetes/hypertension/CKD rather than all 7 comorbidities,
with separate hospitalisation and death cohorts.

- 12_core3_condition_specific_rr.R: mutually-adjusted per-condition RR,
  8-way mutually-exclusive joint-profile RR (pooled, by 5-year age band, and
  as a continuous age curve via factor-smooth GAMs), and an age-interaction
  sensitivity check against the age-invariant-OR assumption.
- 13_core3_descriptive.R: attrition flow, DM/HTN/CKD missingness by age,
  and Table 1 for both cohorts (marginal vs mutually-exclusive framing).
- 14_condition_recording_patterns.R: comorbidity-field recording completeness
  by outcome, age, sex, year, region and state.
- PIPELINE.md: documents the new branch (section 3a).
</commit_message>
<xml_diff>
--- a/CHIK_MORBID/03_Output/tables/chik_sinan_descriptive_tables.xlsx
+++ b/CHIK_MORBID/03_Output/tables/chik_sinan_descriptive_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lshtm-my.sharepoint.com/personal/lsh1800717_lshtm_ac_uk/Documents/Documents/GitHub/CHIK_MORBID/CHIK_MORBID/03_Output/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_438A93DBA52B859C3DB77D8328E87E42B009879C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08C83BC6-51AE-48AE-9EBF-8F97152905EB}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_438A93DBA52B859C3DB77D8328E87E42B009879C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A5C5847-842A-46F4-B3F2-49ED6CC1EB37}"/>
   <bookViews>
-    <workbookView xWindow="375" yWindow="1050" windowWidth="28425" windowHeight="14430" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1260" yWindow="1290" windowWidth="25785" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table1_baseline" sheetId="1" r:id="rId1"/>
@@ -1238,6 +1238,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1709,6 +1719,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -2203,6 +2222,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>